<commit_message>
[auto] session sync 2026-07-22T07:59:24Z
</commit_message>
<xml_diff>
--- a/2D 자동 제작도 개발 현황_2026-07-22.xlsx
+++ b/2D 자동 제작도 개발 현황_2026-07-22.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현황 요약" sheetId="1" r:id="R6152f3530f474ef1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개발 항목" sheetId="2" r:id="Ra63b15680ff740af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항·UDA" sheetId="3" r:id="R63917df2208c46e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="현황 요약" sheetId="1" r:id="R27ef5c8373c64324"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개발 항목" sheetId="2" r:id="Re97d0ad7e26748ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요구사항·UDA" sheetId="3" r:id="R4436b9402c4e43ce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -69,9 +69,6 @@
     <x:t xml:space="preserve">가공도·4종 일괄 차단</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">벤더 수정/회신 후 재검증</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">가공도 캡처 경로</x:t>
   </x:si>
   <x:si>
@@ -108,6 +105,9 @@
     <x:t xml:space="preserve">2D 모서리·홀·실선/은선 누락</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">API 대기</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">형상 누락</x:t>
   </x:si>
   <x:si>
@@ -438,6 +438,21 @@
     <x:t xml:space="preserve">일부 부재 재발 사례와 실선·은선 누락 존재</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">레이아웃·표현</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">가공도 EA 부재 출력 크기·실선/은선·치수 풍선 위치</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">EA 두 뷰 축척 정합, 실선/은선 누락, 치수 풍선 근접 배치</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">API 보강</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">EA 부재의 두 뷰 크기와 선 표현을 맞추고, 치수 풍선을 측정 대상 가까운 영역에 배치하기 위한 항목</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">단면 위주 출력·은선 정책</x:t>
   </x:si>
   <x:si>
@@ -501,6 +516,18 @@
     <x:t xml:space="preserve">정식 필드명과 데이터 소스 확정 필요</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">ISO 풍선 API</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">ISO 풍선 배치 영역 고정 API</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">현재 3D 오프셋 + 2D AABB 충돌 회피만 있고 배치 영역 지정 API는 없음</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">풍선을 지정 영역 안에 고정하면서 측정 대상 가까이 배치할 수 있는 API 필요</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">Tag No</x:t>
   </x:si>
   <x:si>
@@ -627,6 +654,18 @@
     <x:t xml:space="preserve">접합 위치·연결 치수 코드 완료, 최종 PDF 검증 대기</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">템플릿 API</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">빈 셀 테두리 삭제 시 고정 템플릿 테두리 보존</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">RemoveEmptyTemplateBorders 사용 시 고정 템플릿 테두리까지 삭제됨</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">빈 셀 테두리만 삭제하고 도면 양식의 고정 테두리는 유지하도록 API 개선 필요</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">BOM 디자인</x:t>
   </x:si>
   <x:si>
@@ -1008,6 +1047,27 @@
     <x:t xml:space="preserve">Excel 템플릿·직접 그리기·예외 경로에 공통 적용하고 2D 객체는 유지; 연속 출력 실기 확인 대기</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">템플릿 Input 다량 적용 시 보호된 메모리 충돌</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">일부 템플릿에서 Input 항목이 많아지면 적용 중 보호된 메모리 접근 충돌 발생</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">API 수정</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">대량 Input에서도 충돌 없이 템플릿을 적용할 수 있도록 API 안정화 필요</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">템플릿 텍스트 Bold 적용 API</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">템플릿 출력 시 특정 텍스트의 Bold 속성을 코드에서 지정할 수 없음</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">도면 제목·표제부 등 선택 텍스트에 Bold를 적용할 수 있는 API 필요</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">도면 요구사항과 현재 UDA·API 매핑</x:t>
   </x:si>
   <x:si>
@@ -1041,7 +1101,7 @@
     <x:t xml:space="preserve">ISO_PLUS</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">ISO3는 ISO_PLUS 뷰로 확정</x:t>
+    <x:t xml:space="preserve">View_1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">평면도</x:t>
@@ -1363,9 +1423,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="1">
     <x:numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
   <x:fonts count="14">
     <x:font>
@@ -1682,7 +1741,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="49">
+  <x:cellXfs count="43">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -1712,9 +1771,6 @@
     </x:xf>
     <x:xf numFmtId="176" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
@@ -1758,6 +1814,18 @@
     <x:xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center"/>
     </x:xf>
@@ -1765,9 +1833,6 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1">
@@ -1800,41 +1865,61 @@
     <x:xf numFmtId="0" fontId="8" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <x:xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="200" fontId="13" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="표준" xfId="0"/>
   </x:cellStyles>
   <x:dxfs count="18">
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFF4CCCC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF333333"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE7E6E6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
     <x:dxf>
       <x:font>
         <x:b/>
@@ -1915,6 +2000,39 @@
     <x:dxf>
       <x:font>
         <x:b/>
+        <x:color rgb="FF1F4E78"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDEBF7"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFFFF2CC"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF006100"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill>
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
@@ -1956,89 +2074,12 @@
         </x:patternFill>
       </x:fill>
     </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF006100"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE2F0D9"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C6500"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFFF2CC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF1F4E78"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFDDEBF7"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFCE4D6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF333333"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFE7E6E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:font>
-        <x:b/>
-        <x:color rgb="FF9C0006"/>
-      </x:font>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4CCCC"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
   </x:dxfs>
 </x:styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DrawingDevelopmentStatus" displayName="DrawingDevelopmentStatus" ref="A5:Q76" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DrawingDevelopmentStatus" displayName="DrawingDevelopmentStatus" ref="A5:Q76" totalsRowShown="0">
   <x:autoFilter ref="A5:Q76"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="No."/>
@@ -2270,30 +2311,30 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34.04999923706055" customHeight="1">
-      <x:c r="A1" s="11" t="s">
+      <x:c r="A1" s="10" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="11"/>
-      <x:c r="C1" s="11"/>
-      <x:c r="D1" s="11"/>
-      <x:c r="E1" s="11"/>
-      <x:c r="F1" s="11"/>
-      <x:c r="G1" s="11"/>
-      <x:c r="H1" s="11"/>
+      <x:c r="B1" s="10"/>
+      <x:c r="C1" s="10"/>
+      <x:c r="D1" s="10"/>
+      <x:c r="E1" s="10"/>
+      <x:c r="F1" s="10"/>
+      <x:c r="G1" s="10"/>
+      <x:c r="H1" s="10"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="12" t="s">
+      <x:c r="A2" s="11" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B2" s="12"/>
-      <x:c r="C2" s="12"/>
-      <x:c r="D2" s="12"/>
-      <x:c r="E2" s="12"/>
-      <x:c r="F2" s="12"/>
-      <x:c r="G2" s="12"/>
-      <x:c r="H2" s="12"/>
-    </x:row>
-    <x:row r="3" ht="18.600000381469727">
+      <x:c r="B2" s="11"/>
+      <x:c r="C2" s="11"/>
+      <x:c r="D2" s="11"/>
+      <x:c r="E2" s="11"/>
+      <x:c r="F2" s="11"/>
+      <x:c r="G2" s="11"/>
+      <x:c r="H2" s="11"/>
+    </x:row>
+    <x:row r="3">
       <x:c r="A3"/>
       <x:c r="B3"/>
       <x:c r="C3"/>
@@ -2301,55 +2342,55 @@
       <x:c r="E3"/>
       <x:c r="F3"/>
     </x:row>
-    <x:row r="4" ht="18.600000381469727">
-      <x:c r="A4" s="13" t="s">
+    <x:row r="4">
+      <x:c r="A4" s="12" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B4" s="14"/>
-      <x:c r="C4" s="19" t="s">
+      <x:c r="B4" s="13"/>
+      <x:c r="C4" s="18" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="D4" s="20"/>
-      <x:c r="E4" s="21" t="s">
+      <x:c r="D4" s="19"/>
+      <x:c r="E4" s="20" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="F4" s="22"/>
-      <x:c r="G4" s="23" t="s">
+      <x:c r="F4" s="21"/>
+      <x:c r="G4" s="22" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="H4" s="24"/>
+      <x:c r="H4" s="23"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="15" t="n">
+      <x:c r="A5" s="14" t="n">
         <x:f>COUNTA('개발 항목'!$D$6:$D$76)</x:f>
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B5" s="16"/>
-      <x:c r="C5" s="15" t="n">
+      <x:c r="B5" s="15"/>
+      <x:c r="C5" s="14" t="n">
         <x:f>COUNTIF('개발 항목'!$I$6:$I$76,"완료")</x:f>
         <x:v>24</x:v>
       </x:c>
-      <x:c r="D5" s="16"/>
-      <x:c r="E5" s="15" t="n">
+      <x:c r="D5" s="15"/>
+      <x:c r="E5" s="14" t="n">
         <x:f>COUNTIF('개발 항목'!$I$6:$I$76,"실기 검증 대기")</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="F5" s="16"/>
-      <x:c r="G5" s="15" t="n">
+      <x:c r="F5" s="15"/>
+      <x:c r="G5" s="14" t="n">
         <x:f>COUNTIFS('개발 항목'!$E$6:$E$76,"○",'개발 항목'!$H$6:$H$76,"&lt;&gt;O")</x:f>
         <x:v>36</x:v>
       </x:c>
-      <x:c r="H5" s="16"/>
-    </x:row>
-    <x:row r="6" ht="18.600000381469727">
-      <x:c r="A6" s="17"/>
-      <x:c r="B6" s="18"/>
-      <x:c r="C6" s="17"/>
-      <x:c r="D6" s="18"/>
-      <x:c r="E6" s="17"/>
-      <x:c r="F6" s="18"/>
-      <x:c r="G6" s="17"/>
-      <x:c r="H6" s="18"/>
+      <x:c r="H5" s="15"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="16"/>
+      <x:c r="B6" s="17"/>
+      <x:c r="C6" s="16"/>
+      <x:c r="D6" s="17"/>
+      <x:c r="E6" s="16"/>
+      <x:c r="F6" s="17"/>
+      <x:c r="G6" s="16"/>
+      <x:c r="H6" s="17"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7"/>
@@ -2360,16 +2401,16 @@
       <x:c r="F7"/>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="42" t="s">
+      <x:c r="A8" s="27" t="s">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B8" s="42"/>
-      <x:c r="C8" s="42"/>
-      <x:c r="D8" s="42"/>
-      <x:c r="E8" s="42"/>
-      <x:c r="F8" s="42"/>
-      <x:c r="G8" s="42"/>
-      <x:c r="H8" s="42"/>
+      <x:c r="B8" s="27"/>
+      <x:c r="C8" s="27"/>
+      <x:c r="D8" s="27"/>
+      <x:c r="E8" s="27"/>
+      <x:c r="F8" s="27"/>
+      <x:c r="G8" s="27"/>
+      <x:c r="H8" s="27"/>
     </x:row>
     <x:row r="9" ht="18" customHeight="1">
       <x:c r="A9" s="6" t="s">
@@ -2413,11 +2454,11 @@
       <x:c r="E10" s="7" t="s">
         <x:v>18</x:v>
       </x:c>
-      <x:c r="F10" s="7" t="s">
+      <x:c r="F10" s="7" t="str">
+        <x:v>API 수정 후 재검증</x:v>
+      </x:c>
+      <x:c r="G10" s="7" t="s">
         <x:v>19</x:v>
-      </x:c>
-      <x:c r="G10" s="7" t="s">
-        <x:v>20</x:v>
       </x:c>
       <x:c r="H10" s="9">
         <x:v>46224</x:v>
@@ -2428,22 +2469,22 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C11" s="7" t="s">
         <x:v>21</x:v>
-      </x:c>
-      <x:c r="C11" s="7" t="s">
-        <x:v>22</x:v>
       </x:c>
       <x:c r="D11" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E11" s="7" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F11" s="7" t="s">
         <x:v>23</x:v>
       </x:c>
-      <x:c r="F11" s="7" t="s">
+      <x:c r="G11" s="7" t="s">
         <x:v>24</x:v>
-      </x:c>
-      <x:c r="G11" s="7" t="s">
-        <x:v>25</x:v>
       </x:c>
       <x:c r="H11" s="9">
         <x:v>46224</x:v>
@@ -2454,22 +2495,22 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C12" s="7" t="s">
         <x:v>26</x:v>
-      </x:c>
-      <x:c r="C12" s="7" t="s">
-        <x:v>27</x:v>
       </x:c>
       <x:c r="D12" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="E12" s="7" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F12" s="7" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F12" s="7" t="s">
+      <x:c r="G12" s="7" t="s">
         <x:v>29</x:v>
-      </x:c>
-      <x:c r="G12" s="7" t="s">
-        <x:v>30</x:v>
       </x:c>
       <x:c r="H12" s="9">
         <x:v>46225</x:v>
@@ -2480,13 +2521,13 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C13" s="7" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D13" s="8" t="s">
         <x:v>31</x:v>
-      </x:c>
-      <x:c r="D13" s="8" t="str">
-        <x:v>API 대기</x:v>
       </x:c>
       <x:c r="E13" s="7" t="s">
         <x:v>32</x:v>
@@ -2511,8 +2552,8 @@
       <x:c r="C14" s="7" t="s">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="D14" s="8" t="str">
-        <x:v>API 대기</x:v>
+      <x:c r="D14" s="8" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E14" s="7" t="s">
         <x:v>36</x:v>
@@ -2584,7 +2625,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C17" s="7" t="s">
         <x:v>50</x:v>
@@ -2640,89 +2681,96 @@
       <x:c r="F19"/>
     </x:row>
     <x:row r="20" ht="18" customHeight="1">
-      <x:c r="A20" s="42" t="s">
+      <x:c r="A20" s="27" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="B20" s="42"/>
-      <x:c r="C20" s="42"/>
-      <x:c r="D20" s="42"/>
-      <x:c r="E20" s="42"/>
-      <x:c r="F20" s="42"/>
-      <x:c r="G20" s="42"/>
-      <x:c r="H20" s="42"/>
+      <x:c r="B20" s="27"/>
+      <x:c r="C20" s="27"/>
+      <x:c r="D20" s="27"/>
+      <x:c r="E20" s="27"/>
+      <x:c r="F20" s="27"/>
+      <x:c r="G20" s="27"/>
+      <x:c r="H20" s="27"/>
     </x:row>
     <x:row r="21" ht="30" customHeight="1">
       <x:c r="A21" s="4" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B21" s="39" t="s">
+      <x:c r="B21" s="24" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="C21" s="40"/>
-      <x:c r="D21" s="40"/>
-      <x:c r="E21" s="40"/>
-      <x:c r="F21" s="40"/>
-      <x:c r="G21" s="40"/>
-      <x:c r="H21" s="41"/>
+      <x:c r="C21" s="25"/>
+      <x:c r="D21" s="25"/>
+      <x:c r="E21" s="25"/>
+      <x:c r="F21" s="25"/>
+      <x:c r="G21" s="25"/>
+      <x:c r="H21" s="26"/>
     </x:row>
     <x:row r="22" ht="30" customHeight="1">
       <x:c r="A22" s="4" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="B22" s="39" t="s">
+      <x:c r="B22" s="24" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="C22" s="40"/>
-      <x:c r="D22" s="40"/>
-      <x:c r="E22" s="40"/>
-      <x:c r="F22" s="40"/>
-      <x:c r="G22" s="40"/>
-      <x:c r="H22" s="41"/>
+      <x:c r="C22" s="25"/>
+      <x:c r="D22" s="25"/>
+      <x:c r="E22" s="25"/>
+      <x:c r="F22" s="25"/>
+      <x:c r="G22" s="25"/>
+      <x:c r="H22" s="26"/>
     </x:row>
     <x:row r="23" ht="30" customHeight="1">
       <x:c r="A23" s="4" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="B23" s="39" t="s">
+      <x:c r="B23" s="24" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="C23" s="40"/>
-      <x:c r="D23" s="40"/>
-      <x:c r="E23" s="40"/>
-      <x:c r="F23" s="40"/>
-      <x:c r="G23" s="40"/>
-      <x:c r="H23" s="41"/>
+      <x:c r="C23" s="25"/>
+      <x:c r="D23" s="25"/>
+      <x:c r="E23" s="25"/>
+      <x:c r="F23" s="25"/>
+      <x:c r="G23" s="25"/>
+      <x:c r="H23" s="26"/>
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="4" t="s">
         <x:v>68</x:v>
       </x:c>
-      <x:c r="B24" s="39" t="s">
+      <x:c r="B24" s="24" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C24" s="40"/>
-      <x:c r="D24" s="40"/>
-      <x:c r="E24" s="40"/>
-      <x:c r="F24" s="40"/>
-      <x:c r="G24" s="40"/>
-      <x:c r="H24" s="41"/>
+      <x:c r="C24" s="25"/>
+      <x:c r="D24" s="25"/>
+      <x:c r="E24" s="25"/>
+      <x:c r="F24" s="25"/>
+      <x:c r="G24" s="25"/>
+      <x:c r="H24" s="26"/>
     </x:row>
     <x:row r="25" ht="30" customHeight="1">
       <x:c r="A25" s="4" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="B25" s="39" t="s">
+      <x:c r="B25" s="24" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="C25" s="40"/>
-      <x:c r="D25" s="40"/>
-      <x:c r="E25" s="40"/>
-      <x:c r="F25" s="40"/>
-      <x:c r="G25" s="40"/>
-      <x:c r="H25" s="41"/>
+      <x:c r="C25" s="25"/>
+      <x:c r="D25" s="25"/>
+      <x:c r="E25" s="25"/>
+      <x:c r="F25" s="25"/>
+      <x:c r="G25" s="25"/>
+      <x:c r="H25" s="26"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
+    <x:mergeCell ref="B24:H24"/>
+    <x:mergeCell ref="B25:H25"/>
+    <x:mergeCell ref="A8:H8"/>
+    <x:mergeCell ref="A20:H20"/>
+    <x:mergeCell ref="B22:H22"/>
+    <x:mergeCell ref="B23:H23"/>
+    <x:mergeCell ref="B21:H21"/>
     <x:mergeCell ref="A1:H1"/>
     <x:mergeCell ref="A2:H2"/>
     <x:mergeCell ref="A4:B4"/>
@@ -2733,13 +2781,6 @@
     <x:mergeCell ref="E5:F6"/>
     <x:mergeCell ref="G4:H4"/>
     <x:mergeCell ref="G5:H6"/>
-    <x:mergeCell ref="B24:H24"/>
-    <x:mergeCell ref="B25:H25"/>
-    <x:mergeCell ref="A8:H8"/>
-    <x:mergeCell ref="A20:H20"/>
-    <x:mergeCell ref="B22:H22"/>
-    <x:mergeCell ref="B23:H23"/>
-    <x:mergeCell ref="B21:H21"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2767,70 +2808,70 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34.04999923706055" customHeight="1">
-      <x:c r="A1" s="25" t="s">
+      <x:c r="A1" s="28" t="s">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="B1" s="25"/>
-      <x:c r="C1" s="25"/>
-      <x:c r="D1" s="25"/>
-      <x:c r="E1" s="25"/>
-      <x:c r="F1" s="25"/>
-      <x:c r="G1" s="25"/>
-      <x:c r="H1" s="25"/>
-      <x:c r="I1" s="25"/>
-      <x:c r="J1" s="25"/>
-      <x:c r="K1" s="25"/>
-      <x:c r="L1" s="25"/>
-      <x:c r="M1" s="25"/>
-      <x:c r="N1" s="25"/>
-      <x:c r="O1" s="25"/>
-      <x:c r="P1" s="25"/>
-      <x:c r="Q1" s="25"/>
-      <x:c r="R1" s="25"/>
+      <x:c r="B1" s="28"/>
+      <x:c r="C1" s="28"/>
+      <x:c r="D1" s="28"/>
+      <x:c r="E1" s="28"/>
+      <x:c r="F1" s="28"/>
+      <x:c r="G1" s="28"/>
+      <x:c r="H1" s="28"/>
+      <x:c r="I1" s="28"/>
+      <x:c r="J1" s="28"/>
+      <x:c r="K1" s="28"/>
+      <x:c r="L1" s="28"/>
+      <x:c r="M1" s="28"/>
+      <x:c r="N1" s="28"/>
+      <x:c r="O1" s="28"/>
+      <x:c r="P1" s="28"/>
+      <x:c r="Q1" s="28"/>
+      <x:c r="R1" s="28"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="26" t="s">
+      <x:c r="A2" s="29" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="B2" s="26"/>
-      <x:c r="C2" s="26"/>
-      <x:c r="D2" s="26"/>
-      <x:c r="E2" s="26"/>
-      <x:c r="F2" s="26"/>
-      <x:c r="G2" s="26"/>
-      <x:c r="H2" s="26"/>
-      <x:c r="I2" s="26"/>
-      <x:c r="J2" s="26"/>
-      <x:c r="K2" s="26"/>
-      <x:c r="L2" s="26"/>
-      <x:c r="M2" s="26"/>
-      <x:c r="N2" s="26"/>
-      <x:c r="O2" s="26"/>
-      <x:c r="P2" s="26"/>
-      <x:c r="Q2" s="26"/>
-      <x:c r="R2" s="26"/>
+      <x:c r="B2" s="29"/>
+      <x:c r="C2" s="29"/>
+      <x:c r="D2" s="29"/>
+      <x:c r="E2" s="29"/>
+      <x:c r="F2" s="29"/>
+      <x:c r="G2" s="29"/>
+      <x:c r="H2" s="29"/>
+      <x:c r="I2" s="29"/>
+      <x:c r="J2" s="29"/>
+      <x:c r="K2" s="29"/>
+      <x:c r="L2" s="29"/>
+      <x:c r="M2" s="29"/>
+      <x:c r="N2" s="29"/>
+      <x:c r="O2" s="29"/>
+      <x:c r="P2" s="29"/>
+      <x:c r="Q2" s="29"/>
+      <x:c r="R2" s="29"/>
     </x:row>
     <x:row r="3">
-      <x:c r="A3" s="27" t="s">
+      <x:c r="A3" s="30" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="B3" s="27"/>
-      <x:c r="C3" s="27"/>
-      <x:c r="D3" s="27"/>
-      <x:c r="E3" s="27"/>
-      <x:c r="F3" s="27"/>
-      <x:c r="G3" s="27"/>
-      <x:c r="H3" s="27"/>
-      <x:c r="I3" s="27"/>
-      <x:c r="J3" s="27"/>
-      <x:c r="K3" s="27"/>
-      <x:c r="L3" s="27"/>
-      <x:c r="M3" s="27"/>
-      <x:c r="N3" s="27"/>
-      <x:c r="O3" s="27"/>
-      <x:c r="P3" s="27"/>
-      <x:c r="Q3" s="27"/>
-      <x:c r="R3" s="27"/>
+      <x:c r="B3" s="30"/>
+      <x:c r="C3" s="30"/>
+      <x:c r="D3" s="30"/>
+      <x:c r="E3" s="30"/>
+      <x:c r="F3" s="30"/>
+      <x:c r="G3" s="30"/>
+      <x:c r="H3" s="30"/>
+      <x:c r="I3" s="30"/>
+      <x:c r="J3" s="30"/>
+      <x:c r="K3" s="30"/>
+      <x:c r="L3" s="30"/>
+      <x:c r="M3" s="30"/>
+      <x:c r="N3" s="30"/>
+      <x:c r="O3" s="30"/>
+      <x:c r="P3" s="30"/>
+      <x:c r="Q3" s="30"/>
+      <x:c r="R3" s="30"/>
     </x:row>
     <x:row r="5" ht="43.95000076293945" customHeight="1">
       <x:c r="A5" s="6" t="s">
@@ -3193,7 +3234,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B12" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C12" s="8" t="s">
         <x:v>118</x:v>
@@ -3247,7 +3288,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B13" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C13" s="8" t="s">
         <x:v>118</x:v>
@@ -3457,7 +3498,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B17" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C17" s="8" t="s">
         <x:v>137</x:v>
@@ -3477,8 +3518,8 @@
       <x:c r="H17" s="8" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="I17" s="8" t="str">
-        <x:v>API 대기</x:v>
+      <x:c r="I17" s="8" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="J17" s="7" t="s">
         <x:v>139</x:v>
@@ -3508,51 +3549,51 @@
       <x:c r="A18" s="8">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="B18" s="8" t="str">
-        <x:v>가공도</x:v>
-      </x:c>
-      <x:c r="C18" s="8" t="str">
-        <x:v>레이아웃·표현</x:v>
-      </x:c>
-      <x:c r="D18" s="7" t="str">
-        <x:v>가공도 EA 부재 출력 크기·실선/은선·치수 풍선 위치</x:v>
-      </x:c>
-      <x:c r="E18" s="8" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="F18" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G18" s="8" t="str">
-        <x:v>△</x:v>
-      </x:c>
-      <x:c r="H18" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I18" s="8" t="str">
-        <x:v>API 대기</x:v>
-      </x:c>
-      <x:c r="J18" s="7" t="str">
-        <x:v>EA 두 뷰 축척 정합, 실선/은선 누락, 치수 풍선 근접 배치</x:v>
-      </x:c>
-      <x:c r="K18" s="8" t="str">
-        <x:v>API 보강</x:v>
-      </x:c>
-      <x:c r="L18" s="8" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="M18" s="8" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="N18" s="9" t="n">
+      <x:c r="B18" s="8" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C18" s="8" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="D18" s="7" t="s">
+        <x:v>143</x:v>
+      </x:c>
+      <x:c r="E18" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="F18" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G18" s="8" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="H18" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I18" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J18" s="7" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="K18" s="8" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="L18" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="M18" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="N18" s="9">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O18" s="9"/>
-      <x:c r="P18" s="9" t="n">
+      <x:c r="P18" s="9">
         <x:v>46225</x:v>
       </x:c>
-      <x:c r="Q18" s="7" t="str">
-        <x:v>EA 부재의 두 뷰 크기와 선 표현을 맞추고, 치수 풍선을 측정 대상 가까운 영역에 배치하기 위한 항목</x:v>
+      <x:c r="Q18" s="7" t="s">
+        <x:v>146</x:v>
       </x:c>
       <x:c r="R18"/>
     </x:row>
@@ -3567,7 +3608,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D19" s="7" t="s">
-        <x:v>142</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="E19" s="8" t="s">
         <x:v>94</x:v>
@@ -3581,11 +3622,11 @@
       <x:c r="H19" s="8" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="I19" s="8" t="str">
-        <x:v>API 대기</x:v>
+      <x:c r="I19" s="8" t="s">
+        <x:v>31</x:v>
       </x:c>
       <x:c r="J19" s="7" t="s">
-        <x:v>143</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="K19" s="8" t="s">
         <x:v>140</x:v>
@@ -3604,7 +3645,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q19" s="7" t="s">
-        <x:v>144</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="R19"/>
     </x:row>
@@ -3613,13 +3654,13 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B20" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C20" s="8" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D20" s="7" t="s">
-        <x:v>145</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="E20" s="8" t="s">
         <x:v>94</x:v>
@@ -3637,7 +3678,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="J20" s="7" t="s">
-        <x:v>146</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="K20" s="8" t="s">
         <x:v>97</x:v>
@@ -3656,7 +3697,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q20" s="7" t="s">
-        <x:v>147</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="R20"/>
     </x:row>
@@ -3671,7 +3712,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D21" s="7" t="s">
-        <x:v>148</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="E21" s="8" t="s">
         <x:v>94</x:v>
@@ -3689,7 +3730,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="J21" s="7" t="s">
-        <x:v>149</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="K21" s="8" t="s">
         <x:v>97</x:v>
@@ -3708,7 +3749,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q21" s="7" t="s">
-        <x:v>150</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="R21"/>
     </x:row>
@@ -3723,7 +3764,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D22" s="7" t="s">
-        <x:v>151</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="E22" s="8" t="s">
         <x:v>94</x:v>
@@ -3735,16 +3776,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H22" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I22" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J22" s="7" t="s">
-        <x:v>153</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="K22" s="8" t="s">
-        <x:v>154</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="L22" s="8" t="s">
         <x:v>103</x:v>
@@ -3760,7 +3801,7 @@
         <x:v>46155</x:v>
       </x:c>
       <x:c r="Q22" s="7" t="s">
-        <x:v>155</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="R22"/>
     </x:row>
@@ -3775,7 +3816,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D23" s="7" t="s">
-        <x:v>156</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="E23" s="8" t="s">
         <x:v>94</x:v>
@@ -3793,10 +3834,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="J23" s="7" t="s">
-        <x:v>157</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="K23" s="8" t="s">
-        <x:v>158</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="L23" s="8" t="s">
         <x:v>103</x:v>
@@ -3812,7 +3853,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q23" s="7" t="s">
-        <x:v>159</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="R23"/>
     </x:row>
@@ -3827,7 +3868,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D24" s="7" t="s">
-        <x:v>160</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="E24" s="8" t="s">
         <x:v>94</x:v>
@@ -3845,10 +3886,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="J24" s="7" t="s">
-        <x:v>161</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="K24" s="8" t="s">
-        <x:v>158</x:v>
+        <x:v>163</x:v>
       </x:c>
       <x:c r="L24" s="8" t="s">
         <x:v>103</x:v>
@@ -3864,7 +3905,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q24" s="7" t="s">
-        <x:v>162</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="R24"/>
     </x:row>
@@ -3875,48 +3916,48 @@
       <x:c r="B25" s="8" t="s">
         <x:v>133</x:v>
       </x:c>
-      <x:c r="C25" s="8" t="str">
-        <x:v>ISO 풍선 API</x:v>
-      </x:c>
-      <x:c r="D25" s="7" t="str">
-        <x:v>ISO 풍선 배치 영역 고정 API</x:v>
-      </x:c>
-      <x:c r="E25" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F25" s="8" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="G25" s="8" t="str">
-        <x:v>△</x:v>
-      </x:c>
-      <x:c r="H25" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I25" s="8" t="str">
-        <x:v>API 대기</x:v>
-      </x:c>
-      <x:c r="J25" s="7" t="str">
-        <x:v>현재 3D 오프셋 + 2D AABB 충돌 회피만 있고 배치 영역 지정 API는 없음</x:v>
-      </x:c>
-      <x:c r="K25" s="8" t="str">
-        <x:v>API 보강</x:v>
-      </x:c>
-      <x:c r="L25" s="8" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="M25" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="N25" s="9" t="n">
+      <x:c r="C25" s="8" t="s">
+        <x:v>168</x:v>
+      </x:c>
+      <x:c r="D25" s="7" t="s">
+        <x:v>169</x:v>
+      </x:c>
+      <x:c r="E25" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="F25" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G25" s="8" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="H25" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I25" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J25" s="7" t="s">
+        <x:v>170</x:v>
+      </x:c>
+      <x:c r="K25" s="8" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="L25" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="M25" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="N25" s="9">
         <x:v>46154</x:v>
       </x:c>
       <x:c r="O25" s="9"/>
-      <x:c r="P25" s="9" t="n">
+      <x:c r="P25" s="9">
         <x:v>46225</x:v>
       </x:c>
-      <x:c r="Q25" s="7" t="str">
-        <x:v>풍선을 지정 영역 안에 고정하면서 측정 대상 가까이 배치할 수 있는 API 필요</x:v>
+      <x:c r="Q25" s="7" t="s">
+        <x:v>171</x:v>
       </x:c>
       <x:c r="R25"/>
     </x:row>
@@ -3931,7 +3972,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D26" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E26" s="8" t="s">
         <x:v>94</x:v>
@@ -3943,16 +3984,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H26" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I26" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J26" s="7" t="s">
-        <x:v>164</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="K26" s="8" t="s">
-        <x:v>165</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="L26" s="8" t="s">
         <x:v>103</x:v>
@@ -3970,7 +4011,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q26" s="7" t="s">
-        <x:v>166</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="R26"/>
     </x:row>
@@ -3982,10 +4023,10 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="C27" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D27" s="7" t="s">
-        <x:v>168</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="E27" s="8" t="s">
         <x:v>94</x:v>
@@ -3997,16 +4038,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H27" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I27" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J27" s="7" t="s">
-        <x:v>169</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="K27" s="8" t="s">
-        <x:v>170</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="L27" s="8" t="s">
         <x:v>103</x:v>
@@ -4022,7 +4063,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q27" s="7" t="s">
-        <x:v>171</x:v>
+        <x:v>180</x:v>
       </x:c>
       <x:c r="R27"/>
     </x:row>
@@ -4034,10 +4075,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C28" s="8" t="s">
-        <x:v>172</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D28" s="7" t="s">
-        <x:v>173</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="E28" s="8" t="s">
         <x:v>94</x:v>
@@ -4049,16 +4090,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H28" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I28" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J28" s="7" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="K28" s="8" t="s">
         <x:v>174</x:v>
-      </x:c>
-      <x:c r="K28" s="8" t="s">
-        <x:v>165</x:v>
       </x:c>
       <x:c r="L28" s="8" t="s">
         <x:v>103</x:v>
@@ -4074,7 +4115,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q28" s="7" t="s">
-        <x:v>175</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="R28"/>
     </x:row>
@@ -4083,13 +4124,13 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B29" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C29" s="8" t="s">
-        <x:v>176</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="D29" s="7" t="s">
-        <x:v>177</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="E29" s="8" t="s">
         <x:v>94</x:v>
@@ -4107,10 +4148,10 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="J29" s="7" t="s">
-        <x:v>178</x:v>
+        <x:v>187</x:v>
       </x:c>
       <x:c r="K29" s="8" t="s">
-        <x:v>179</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="L29" s="8" t="s">
         <x:v>103</x:v>
@@ -4126,7 +4167,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q29" s="7" t="s">
-        <x:v>180</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="R29"/>
     </x:row>
@@ -4141,7 +4182,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D30" s="7" t="s">
-        <x:v>181</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="E30" s="8" t="s">
         <x:v>94</x:v>
@@ -4159,7 +4200,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J30" s="7" t="s">
-        <x:v>182</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="K30" s="8" t="s">
         <x:v>122</x:v>
@@ -4180,7 +4221,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q30" s="7" t="s">
-        <x:v>183</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="R30"/>
     </x:row>
@@ -4195,7 +4236,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D31" s="7" t="s">
-        <x:v>184</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="E31" s="8" t="s">
         <x:v>94</x:v>
@@ -4213,10 +4254,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J31" s="7" t="s">
-        <x:v>185</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="K31" s="8" t="s">
-        <x:v>186</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="L31" s="8" t="s">
         <x:v>103</x:v>
@@ -4230,7 +4271,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q31" s="7" t="s">
-        <x:v>187</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="R31"/>
     </x:row>
@@ -4242,10 +4283,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C32" s="8" t="s">
-        <x:v>188</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="D32" s="7" t="s">
-        <x:v>189</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="E32" s="8" t="s">
         <x:v>94</x:v>
@@ -4263,10 +4304,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J32" s="7" t="s">
-        <x:v>190</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="K32" s="8" t="s">
-        <x:v>191</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="L32" s="8" t="s">
         <x:v>103</x:v>
@@ -4280,7 +4321,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q32" s="7" t="s">
-        <x:v>192</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="R32"/>
     </x:row>
@@ -4292,10 +4333,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C33" s="8" t="s">
-        <x:v>188</x:v>
+        <x:v>197</x:v>
       </x:c>
       <x:c r="D33" s="7" t="s">
-        <x:v>193</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="E33" s="8" t="s">
         <x:v>94</x:v>
@@ -4313,10 +4354,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J33" s="7" t="s">
-        <x:v>194</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="K33" s="8" t="s">
-        <x:v>191</x:v>
+        <x:v>200</x:v>
       </x:c>
       <x:c r="L33" s="8" t="s">
         <x:v>103</x:v>
@@ -4330,7 +4371,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q33" s="7" t="s">
-        <x:v>195</x:v>
+        <x:v>204</x:v>
       </x:c>
       <x:c r="R33"/>
     </x:row>
@@ -4339,13 +4380,13 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B34" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C34" s="8" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D34" s="7" t="s">
-        <x:v>196</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="E34" s="8" t="s">
         <x:v>94</x:v>
@@ -4357,13 +4398,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H34" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I34" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J34" s="7" t="s">
-        <x:v>197</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="K34" s="8" t="s">
         <x:v>122</x:v>
@@ -4382,7 +4423,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q34" s="7" t="s">
-        <x:v>198</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="R34"/>
     </x:row>
@@ -4391,13 +4432,13 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B35" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C35" s="8" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D35" s="7" t="s">
-        <x:v>199</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="E35" s="8" t="s">
         <x:v>94</x:v>
@@ -4409,13 +4450,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H35" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I35" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J35" s="7" t="s">
-        <x:v>200</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="K35" s="8" t="s">
         <x:v>122</x:v>
@@ -4434,7 +4475,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q35" s="7" t="s">
-        <x:v>201</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="R35"/>
     </x:row>
@@ -4443,13 +4484,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B36" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C36" s="8" t="s">
         <x:v>92</x:v>
       </x:c>
       <x:c r="D36" s="7" t="s">
-        <x:v>202</x:v>
+        <x:v>211</x:v>
       </x:c>
       <x:c r="E36" s="8" t="s">
         <x:v>94</x:v>
@@ -4461,13 +4502,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H36" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I36" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J36" s="7" t="s">
-        <x:v>203</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="K36" s="8" t="s">
         <x:v>122</x:v>
@@ -4486,7 +4527,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q36" s="7" t="s">
-        <x:v>204</x:v>
+        <x:v>213</x:v>
       </x:c>
       <x:c r="R36"/>
     </x:row>
@@ -4495,50 +4536,50 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B37" s="8" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="C37" s="8" t="str">
-        <x:v>템플릿 API</x:v>
-      </x:c>
-      <x:c r="D37" s="7" t="str">
-        <x:v>빈 셀 테두리 삭제 시 고정 템플릿 테두리 보존</x:v>
-      </x:c>
-      <x:c r="E37" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F37" s="8" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="G37" s="8" t="str">
-        <x:v>△</x:v>
-      </x:c>
-      <x:c r="H37" s="8" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I37" s="8" t="str">
-        <x:v>API 대기</x:v>
-      </x:c>
-      <x:c r="J37" s="7" t="str">
-        <x:v>RemoveEmptyTemplateBorders 사용 시 고정 템플릿 테두리까지 삭제됨</x:v>
-      </x:c>
-      <x:c r="K37" s="8" t="str">
-        <x:v>API 보강</x:v>
-      </x:c>
-      <x:c r="L37" s="8" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="M37" s="8" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="N37" s="9" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C37" s="8" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="D37" s="7" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="E37" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="F37" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G37" s="8" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="H37" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I37" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J37" s="7" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="K37" s="8" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="L37" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="M37" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="N37" s="9">
         <x:v>46224</x:v>
       </x:c>
       <x:c r="O37" s="9"/>
-      <x:c r="P37" s="9" t="n">
+      <x:c r="P37" s="9">
         <x:v>46225</x:v>
       </x:c>
-      <x:c r="Q37" s="7" t="str">
-        <x:v>빈 셀 테두리만 삭제하고 도면 양식의 고정 테두리는 유지하도록 API 개선 필요</x:v>
+      <x:c r="Q37" s="7" t="s">
+        <x:v>217</x:v>
       </x:c>
       <x:c r="R37"/>
     </x:row>
@@ -4547,13 +4588,13 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B38" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C38" s="8" t="s">
-        <x:v>205</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="D38" s="7" t="s">
-        <x:v>206</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="E38" s="8" t="s">
         <x:v>95</x:v>
@@ -4565,16 +4606,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H38" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I38" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J38" s="7" t="s">
-        <x:v>207</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="K38" s="8" t="s">
-        <x:v>208</x:v>
+        <x:v>221</x:v>
       </x:c>
       <x:c r="L38" s="8" t="s">
         <x:v>103</x:v>
@@ -4590,7 +4631,7 @@
         <x:v>46155</x:v>
       </x:c>
       <x:c r="Q38" s="7" t="s">
-        <x:v>209</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="R38"/>
     </x:row>
@@ -4599,13 +4640,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B39" s="8" t="s">
-        <x:v>210</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="C39" s="8" t="s">
-        <x:v>211</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="D39" s="7" t="s">
-        <x:v>212</x:v>
+        <x:v>225</x:v>
       </x:c>
       <x:c r="E39" s="8" t="s">
         <x:v>94</x:v>
@@ -4623,7 +4664,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J39" s="7" t="s">
-        <x:v>213</x:v>
+        <x:v>226</x:v>
       </x:c>
       <x:c r="K39" s="8" t="s">
         <x:v>122</x:v>
@@ -4644,7 +4685,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q39" s="7" t="s">
-        <x:v>214</x:v>
+        <x:v>227</x:v>
       </x:c>
       <x:c r="R39"/>
     </x:row>
@@ -4653,13 +4694,13 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B40" s="8" t="s">
-        <x:v>215</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="C40" s="8" t="s">
-        <x:v>211</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="D40" s="7" t="s">
-        <x:v>216</x:v>
+        <x:v>229</x:v>
       </x:c>
       <x:c r="E40" s="8" t="s">
         <x:v>94</x:v>
@@ -4677,7 +4718,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J40" s="7" t="s">
-        <x:v>217</x:v>
+        <x:v>230</x:v>
       </x:c>
       <x:c r="K40" s="8" t="s">
         <x:v>122</x:v>
@@ -4698,7 +4739,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q40" s="7" t="s">
-        <x:v>218</x:v>
+        <x:v>231</x:v>
       </x:c>
       <x:c r="R40"/>
     </x:row>
@@ -4713,7 +4754,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D41" s="7" t="s">
-        <x:v>219</x:v>
+        <x:v>232</x:v>
       </x:c>
       <x:c r="E41" s="8" t="s">
         <x:v>120</x:v>
@@ -4748,7 +4789,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q41" s="7" t="s">
-        <x:v>220</x:v>
+        <x:v>233</x:v>
       </x:c>
       <x:c r="R41"/>
     </x:row>
@@ -4757,13 +4798,13 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B42" s="8" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C42" s="8" t="s">
-        <x:v>211</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="D42" s="7" t="s">
-        <x:v>221</x:v>
+        <x:v>234</x:v>
       </x:c>
       <x:c r="E42" s="8" t="s">
         <x:v>94</x:v>
@@ -4775,13 +4816,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H42" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I42" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J42" s="7" t="s">
-        <x:v>222</x:v>
+        <x:v>235</x:v>
       </x:c>
       <x:c r="K42" s="8" t="s">
         <x:v>122</x:v>
@@ -4800,7 +4841,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q42" s="7" t="s">
-        <x:v>223</x:v>
+        <x:v>236</x:v>
       </x:c>
       <x:c r="R42"/>
     </x:row>
@@ -4809,13 +4850,13 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B43" s="8" t="s">
+        <x:v>237</x:v>
+      </x:c>
+      <x:c r="C43" s="8" t="s">
         <x:v>224</x:v>
       </x:c>
-      <x:c r="C43" s="8" t="s">
-        <x:v>211</x:v>
-      </x:c>
       <x:c r="D43" s="7" t="s">
-        <x:v>225</x:v>
+        <x:v>238</x:v>
       </x:c>
       <x:c r="E43" s="8" t="s">
         <x:v>94</x:v>
@@ -4827,13 +4868,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H43" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I43" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J43" s="7" t="s">
-        <x:v>226</x:v>
+        <x:v>239</x:v>
       </x:c>
       <x:c r="K43" s="8" t="s">
         <x:v>122</x:v>
@@ -4852,7 +4893,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q43" s="7" t="s">
-        <x:v>227</x:v>
+        <x:v>240</x:v>
       </x:c>
       <x:c r="R43"/>
     </x:row>
@@ -4861,13 +4902,13 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B44" s="8" t="s">
-        <x:v>21</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C44" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D44" s="7" t="s">
-        <x:v>228</x:v>
+        <x:v>241</x:v>
       </x:c>
       <x:c r="E44" s="8" t="s">
         <x:v>94</x:v>
@@ -4879,13 +4920,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H44" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I44" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J44" s="7" t="s">
-        <x:v>229</x:v>
+        <x:v>242</x:v>
       </x:c>
       <x:c r="K44" s="8" t="s">
         <x:v>122</x:v>
@@ -4904,7 +4945,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q44" s="7" t="s">
-        <x:v>230</x:v>
+        <x:v>243</x:v>
       </x:c>
       <x:c r="R44"/>
     </x:row>
@@ -4916,10 +4957,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C45" s="8" t="s">
-        <x:v>172</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D45" s="7" t="s">
-        <x:v>231</x:v>
+        <x:v>244</x:v>
       </x:c>
       <x:c r="E45" s="8" t="s">
         <x:v>94</x:v>
@@ -4931,13 +4972,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H45" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I45" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J45" s="7" t="s">
-        <x:v>232</x:v>
+        <x:v>245</x:v>
       </x:c>
       <x:c r="K45" s="8" t="s">
         <x:v>122</x:v>
@@ -4956,7 +4997,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q45" s="7" t="s">
-        <x:v>233</x:v>
+        <x:v>246</x:v>
       </x:c>
       <x:c r="R45"/>
     </x:row>
@@ -4968,10 +5009,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C46" s="8" t="s">
-        <x:v>172</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="D46" s="7" t="s">
-        <x:v>234</x:v>
+        <x:v>247</x:v>
       </x:c>
       <x:c r="E46" s="8" t="s">
         <x:v>94</x:v>
@@ -4983,13 +5024,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H46" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I46" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J46" s="7" t="s">
-        <x:v>235</x:v>
+        <x:v>248</x:v>
       </x:c>
       <x:c r="K46" s="8" t="s">
         <x:v>122</x:v>
@@ -5008,7 +5049,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q46" s="7" t="s">
-        <x:v>236</x:v>
+        <x:v>249</x:v>
       </x:c>
       <x:c r="R46"/>
     </x:row>
@@ -5020,10 +5061,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C47" s="8" t="s">
-        <x:v>237</x:v>
+        <x:v>250</x:v>
       </x:c>
       <x:c r="D47" s="7" t="s">
-        <x:v>238</x:v>
+        <x:v>251</x:v>
       </x:c>
       <x:c r="E47" s="8" t="s">
         <x:v>94</x:v>
@@ -5035,16 +5076,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H47" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I47" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J47" s="7" t="s">
-        <x:v>239</x:v>
+        <x:v>252</x:v>
       </x:c>
       <x:c r="K47" s="8" t="s">
-        <x:v>179</x:v>
+        <x:v>188</x:v>
       </x:c>
       <x:c r="L47" s="8" t="s">
         <x:v>103</x:v>
@@ -5060,7 +5101,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q47" s="7" t="s">
-        <x:v>240</x:v>
+        <x:v>253</x:v>
       </x:c>
       <x:c r="R47"/>
     </x:row>
@@ -5075,7 +5116,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D48" s="7" t="s">
-        <x:v>241</x:v>
+        <x:v>254</x:v>
       </x:c>
       <x:c r="E48" s="8" t="s">
         <x:v>94</x:v>
@@ -5093,7 +5134,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J48" s="7" t="s">
-        <x:v>242</x:v>
+        <x:v>255</x:v>
       </x:c>
       <x:c r="K48" s="8" t="s">
         <x:v>122</x:v>
@@ -5112,7 +5153,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q48" s="7" t="s">
-        <x:v>243</x:v>
+        <x:v>256</x:v>
       </x:c>
       <x:c r="R48"/>
     </x:row>
@@ -5127,7 +5168,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="D49" s="7" t="s">
-        <x:v>244</x:v>
+        <x:v>257</x:v>
       </x:c>
       <x:c r="E49" s="8" t="s">
         <x:v>120</x:v>
@@ -5145,7 +5186,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J49" s="7" t="s">
-        <x:v>245</x:v>
+        <x:v>258</x:v>
       </x:c>
       <x:c r="K49" s="8" t="s">
         <x:v>122</x:v>
@@ -5164,7 +5205,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q49" s="7" t="s">
-        <x:v>246</x:v>
+        <x:v>259</x:v>
       </x:c>
       <x:c r="R49"/>
     </x:row>
@@ -5176,10 +5217,10 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="C50" s="8" t="s">
-        <x:v>247</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D50" s="7" t="s">
-        <x:v>248</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="E50" s="8" t="s">
         <x:v>95</x:v>
@@ -5197,7 +5238,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J50" s="7" t="s">
-        <x:v>249</x:v>
+        <x:v>262</x:v>
       </x:c>
       <x:c r="K50" s="8" t="s">
         <x:v>122</x:v>
@@ -5218,7 +5259,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q50" s="7" t="s">
-        <x:v>250</x:v>
+        <x:v>263</x:v>
       </x:c>
       <x:c r="R50"/>
     </x:row>
@@ -5230,10 +5271,10 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="C51" s="8" t="s">
-        <x:v>247</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D51" s="7" t="s">
-        <x:v>251</x:v>
+        <x:v>264</x:v>
       </x:c>
       <x:c r="E51" s="8" t="s">
         <x:v>95</x:v>
@@ -5245,16 +5286,16 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="H51" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I51" s="8" t="s">
         <x:v>57</x:v>
       </x:c>
       <x:c r="J51" s="7" t="s">
-        <x:v>252</x:v>
+        <x:v>265</x:v>
       </x:c>
       <x:c r="K51" s="8" t="s">
-        <x:v>253</x:v>
+        <x:v>266</x:v>
       </x:c>
       <x:c r="L51" s="8" t="s">
         <x:v>103</x:v>
@@ -5270,7 +5311,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q51" s="7" t="s">
-        <x:v>254</x:v>
+        <x:v>267</x:v>
       </x:c>
       <x:c r="R51"/>
     </x:row>
@@ -5282,10 +5323,10 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="C52" s="8" t="s">
-        <x:v>247</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D52" s="7" t="s">
-        <x:v>255</x:v>
+        <x:v>268</x:v>
       </x:c>
       <x:c r="E52" s="8" t="s">
         <x:v>95</x:v>
@@ -5303,7 +5344,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J52" s="7" t="s">
-        <x:v>256</x:v>
+        <x:v>269</x:v>
       </x:c>
       <x:c r="K52" s="8" t="s">
         <x:v>122</x:v>
@@ -5324,7 +5365,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q52" s="7" t="s">
-        <x:v>257</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="R52"/>
     </x:row>
@@ -5336,10 +5377,10 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="C53" s="8" t="s">
-        <x:v>247</x:v>
+        <x:v>260</x:v>
       </x:c>
       <x:c r="D53" s="7" t="s">
-        <x:v>258</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="E53" s="8" t="s">
         <x:v>95</x:v>
@@ -5357,7 +5398,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J53" s="7" t="s">
-        <x:v>259</x:v>
+        <x:v>272</x:v>
       </x:c>
       <x:c r="K53" s="8" t="s">
         <x:v>122</x:v>
@@ -5376,7 +5417,7 @@
         <x:v>46223</x:v>
       </x:c>
       <x:c r="Q53" s="7" t="s">
-        <x:v>260</x:v>
+        <x:v>273</x:v>
       </x:c>
       <x:c r="R53"/>
     </x:row>
@@ -5391,7 +5432,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D54" s="7" t="s">
-        <x:v>261</x:v>
+        <x:v>274</x:v>
       </x:c>
       <x:c r="E54" s="8" t="s">
         <x:v>94</x:v>
@@ -5409,7 +5450,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J54" s="7" t="s">
-        <x:v>262</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="K54" s="8" t="s">
         <x:v>122</x:v>
@@ -5428,7 +5469,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q54" s="7" t="s">
-        <x:v>263</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="R54"/>
     </x:row>
@@ -5443,7 +5484,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D55" s="7" t="s">
-        <x:v>264</x:v>
+        <x:v>277</x:v>
       </x:c>
       <x:c r="E55" s="8" t="s">
         <x:v>94</x:v>
@@ -5461,7 +5502,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J55" s="7" t="s">
-        <x:v>265</x:v>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="K55" s="8" t="s">
         <x:v>122</x:v>
@@ -5480,7 +5521,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q55" s="7" t="s">
-        <x:v>263</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="R55"/>
     </x:row>
@@ -5489,13 +5530,13 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B56" s="8" t="s">
-        <x:v>266</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C56" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D56" s="7" t="s">
-        <x:v>267</x:v>
+        <x:v>280</x:v>
       </x:c>
       <x:c r="E56" s="8" t="s">
         <x:v>120</x:v>
@@ -5513,7 +5554,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J56" s="7" t="s">
-        <x:v>268</x:v>
+        <x:v>281</x:v>
       </x:c>
       <x:c r="K56" s="8" t="s">
         <x:v>97</x:v>
@@ -5530,7 +5571,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q56" s="7" t="s">
-        <x:v>269</x:v>
+        <x:v>282</x:v>
       </x:c>
       <x:c r="R56"/>
     </x:row>
@@ -5545,7 +5586,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="D57" s="7" t="s">
-        <x:v>270</x:v>
+        <x:v>283</x:v>
       </x:c>
       <x:c r="E57" s="8" t="s">
         <x:v>94</x:v>
@@ -5563,7 +5604,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J57" s="7" t="s">
-        <x:v>271</x:v>
+        <x:v>284</x:v>
       </x:c>
       <x:c r="K57" s="8" t="s">
         <x:v>122</x:v>
@@ -5582,7 +5623,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q57" s="7" t="s">
-        <x:v>263</x:v>
+        <x:v>276</x:v>
       </x:c>
       <x:c r="R57"/>
     </x:row>
@@ -5591,13 +5632,13 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B58" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C58" s="8" t="s">
-        <x:v>272</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="D58" s="7" t="s">
-        <x:v>273</x:v>
+        <x:v>286</x:v>
       </x:c>
       <x:c r="E58" s="8" t="s">
         <x:v>95</x:v>
@@ -5615,10 +5656,10 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J58" s="7" t="s">
-        <x:v>274</x:v>
+        <x:v>287</x:v>
       </x:c>
       <x:c r="K58" s="8" t="s">
-        <x:v>275</x:v>
+        <x:v>288</x:v>
       </x:c>
       <x:c r="L58" s="8" t="s">
         <x:v>103</x:v>
@@ -5634,7 +5675,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q58" s="7" t="s">
-        <x:v>276</x:v>
+        <x:v>289</x:v>
       </x:c>
       <x:c r="R58"/>
     </x:row>
@@ -5646,10 +5687,10 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="C59" s="8" t="s">
-        <x:v>211</x:v>
+        <x:v>224</x:v>
       </x:c>
       <x:c r="D59" s="7" t="s">
-        <x:v>277</x:v>
+        <x:v>290</x:v>
       </x:c>
       <x:c r="E59" s="8" t="s">
         <x:v>94</x:v>
@@ -5667,7 +5708,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J59" s="7" t="s">
-        <x:v>278</x:v>
+        <x:v>291</x:v>
       </x:c>
       <x:c r="K59" s="8" t="s">
         <x:v>122</x:v>
@@ -5686,7 +5727,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q59" s="7" t="s">
-        <x:v>279</x:v>
+        <x:v>292</x:v>
       </x:c>
       <x:c r="R59"/>
     </x:row>
@@ -5701,7 +5742,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D60" s="7" t="s">
-        <x:v>280</x:v>
+        <x:v>293</x:v>
       </x:c>
       <x:c r="E60" s="8" t="s">
         <x:v>94</x:v>
@@ -5719,7 +5760,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J60" s="7" t="s">
-        <x:v>281</x:v>
+        <x:v>294</x:v>
       </x:c>
       <x:c r="K60" s="8" t="s">
         <x:v>122</x:v>
@@ -5738,7 +5779,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q60" s="7" t="s">
-        <x:v>282</x:v>
+        <x:v>295</x:v>
       </x:c>
       <x:c r="R60"/>
     </x:row>
@@ -5750,10 +5791,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C61" s="8" t="s">
-        <x:v>272</x:v>
+        <x:v>285</x:v>
       </x:c>
       <x:c r="D61" s="7" t="s">
-        <x:v>283</x:v>
+        <x:v>296</x:v>
       </x:c>
       <x:c r="E61" s="8" t="s">
         <x:v>95</x:v>
@@ -5771,7 +5812,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="J61" s="7" t="s">
-        <x:v>284</x:v>
+        <x:v>297</x:v>
       </x:c>
       <x:c r="K61" s="8" t="s">
         <x:v>97</x:v>
@@ -5788,7 +5829,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q61" s="7" t="s">
-        <x:v>285</x:v>
+        <x:v>298</x:v>
       </x:c>
       <x:c r="R61"/>
     </x:row>
@@ -5803,7 +5844,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D62" s="7" t="s">
-        <x:v>286</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="E62" s="8" t="s">
         <x:v>94</x:v>
@@ -5821,7 +5862,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J62" s="7" t="s">
-        <x:v>287</x:v>
+        <x:v>300</x:v>
       </x:c>
       <x:c r="K62" s="8" t="s">
         <x:v>122</x:v>
@@ -5840,7 +5881,7 @@
         <x:v>46156</x:v>
       </x:c>
       <x:c r="Q62" s="7" t="s">
-        <x:v>288</x:v>
+        <x:v>301</x:v>
       </x:c>
       <x:c r="R62"/>
     </x:row>
@@ -5855,7 +5896,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D63" s="7" t="s">
-        <x:v>289</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="E63" s="8" t="s">
         <x:v>94</x:v>
@@ -5873,7 +5914,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J63" s="7" t="s">
-        <x:v>290</x:v>
+        <x:v>303</x:v>
       </x:c>
       <x:c r="K63" s="8" t="s">
         <x:v>122</x:v>
@@ -5892,7 +5933,7 @@
         <x:v>46155</x:v>
       </x:c>
       <x:c r="Q63" s="7" t="s">
-        <x:v>291</x:v>
+        <x:v>304</x:v>
       </x:c>
       <x:c r="R63"/>
     </x:row>
@@ -5907,7 +5948,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D64" s="7" t="s">
-        <x:v>292</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="E64" s="8" t="s">
         <x:v>94</x:v>
@@ -5925,7 +5966,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J64" s="7" t="s">
-        <x:v>293</x:v>
+        <x:v>306</x:v>
       </x:c>
       <x:c r="K64" s="8" t="s">
         <x:v>122</x:v>
@@ -5944,7 +5985,7 @@
         <x:v>46155</x:v>
       </x:c>
       <x:c r="Q64" s="7" t="s">
-        <x:v>294</x:v>
+        <x:v>307</x:v>
       </x:c>
       <x:c r="R64"/>
     </x:row>
@@ -5959,7 +6000,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="D65" s="7" t="s">
-        <x:v>295</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="E65" s="8" t="s">
         <x:v>94</x:v>
@@ -5977,7 +6018,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J65" s="7" t="s">
-        <x:v>296</x:v>
+        <x:v>309</x:v>
       </x:c>
       <x:c r="K65" s="8" t="s">
         <x:v>122</x:v>
@@ -5996,7 +6037,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q65" s="7" t="s">
-        <x:v>297</x:v>
+        <x:v>310</x:v>
       </x:c>
       <x:c r="R65"/>
     </x:row>
@@ -6005,13 +6046,13 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B66" s="8" t="s">
-        <x:v>215</x:v>
+        <x:v>228</x:v>
       </x:c>
       <x:c r="C66" s="8" t="s">
         <x:v>39</x:v>
       </x:c>
       <x:c r="D66" s="7" t="s">
-        <x:v>298</x:v>
+        <x:v>311</x:v>
       </x:c>
       <x:c r="E66" s="8" t="s">
         <x:v>94</x:v>
@@ -6029,7 +6070,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J66" s="7" t="s">
-        <x:v>299</x:v>
+        <x:v>312</x:v>
       </x:c>
       <x:c r="K66" s="8" t="s">
         <x:v>122</x:v>
@@ -6050,7 +6091,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q66" s="7" t="s">
-        <x:v>300</x:v>
+        <x:v>313</x:v>
       </x:c>
       <x:c r="R66"/>
     </x:row>
@@ -6059,13 +6100,13 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B67" s="8" t="s">
-        <x:v>266</x:v>
+        <x:v>279</x:v>
       </x:c>
       <x:c r="C67" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D67" s="7" t="s">
-        <x:v>301</x:v>
+        <x:v>314</x:v>
       </x:c>
       <x:c r="E67" s="8" t="s">
         <x:v>94</x:v>
@@ -6083,7 +6124,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J67" s="7" t="s">
-        <x:v>302</x:v>
+        <x:v>315</x:v>
       </x:c>
       <x:c r="K67" s="8" t="s">
         <x:v>122</x:v>
@@ -6104,7 +6145,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q67" s="7" t="s">
-        <x:v>303</x:v>
+        <x:v>316</x:v>
       </x:c>
       <x:c r="R67"/>
     </x:row>
@@ -6116,10 +6157,10 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="C68" s="8" t="s">
-        <x:v>304</x:v>
+        <x:v>317</x:v>
       </x:c>
       <x:c r="D68" s="7" t="s">
-        <x:v>305</x:v>
+        <x:v>318</x:v>
       </x:c>
       <x:c r="E68" s="8" t="s">
         <x:v>95</x:v>
@@ -6131,13 +6172,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H68" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I68" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J68" s="7" t="s">
-        <x:v>306</x:v>
+        <x:v>319</x:v>
       </x:c>
       <x:c r="K68" s="8" t="s">
         <x:v>122</x:v>
@@ -6156,7 +6197,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q68" s="7" t="s">
-        <x:v>307</x:v>
+        <x:v>320</x:v>
       </x:c>
       <x:c r="R68"/>
     </x:row>
@@ -6165,13 +6206,13 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B69" s="8" t="s">
-        <x:v>308</x:v>
+        <x:v>321</x:v>
       </x:c>
       <x:c r="C69" s="8" t="s">
-        <x:v>167</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="D69" s="7" t="s">
-        <x:v>309</x:v>
+        <x:v>322</x:v>
       </x:c>
       <x:c r="E69" s="8" t="s">
         <x:v>94</x:v>
@@ -6189,7 +6230,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J69" s="7" t="s">
-        <x:v>310</x:v>
+        <x:v>323</x:v>
       </x:c>
       <x:c r="K69" s="8" t="s">
         <x:v>122</x:v>
@@ -6210,7 +6251,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q69" s="7" t="s">
-        <x:v>311</x:v>
+        <x:v>324</x:v>
       </x:c>
       <x:c r="R69"/>
     </x:row>
@@ -6219,13 +6260,13 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B70" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C70" s="8" t="s">
-        <x:v>312</x:v>
+        <x:v>325</x:v>
       </x:c>
       <x:c r="D70" s="7" t="s">
-        <x:v>313</x:v>
+        <x:v>326</x:v>
       </x:c>
       <x:c r="E70" s="8" t="s">
         <x:v>95</x:v>
@@ -6237,13 +6278,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H70" s="8" t="s">
-        <x:v>314</x:v>
+        <x:v>327</x:v>
       </x:c>
       <x:c r="I70" s="8" t="s">
         <x:v>3</x:v>
       </x:c>
       <x:c r="J70" s="7" t="s">
-        <x:v>315</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="K70" s="8" t="s">
         <x:v>122</x:v>
@@ -6264,7 +6305,7 @@
         <x:v>46222</x:v>
       </x:c>
       <x:c r="Q70" s="7" t="s">
-        <x:v>316</x:v>
+        <x:v>329</x:v>
       </x:c>
       <x:c r="R70"/>
     </x:row>
@@ -6273,13 +6314,13 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B71" s="8" t="s">
-        <x:v>26</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C71" s="8" t="s">
-        <x:v>317</x:v>
+        <x:v>330</x:v>
       </x:c>
       <x:c r="D71" s="7" t="s">
-        <x:v>318</x:v>
+        <x:v>331</x:v>
       </x:c>
       <x:c r="E71" s="8" t="s">
         <x:v>95</x:v>
@@ -6297,7 +6338,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="J71" s="7" t="s">
-        <x:v>319</x:v>
+        <x:v>332</x:v>
       </x:c>
       <x:c r="K71" s="8" t="s">
         <x:v>122</x:v>
@@ -6318,7 +6359,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q71" s="7" t="s">
-        <x:v>320</x:v>
+        <x:v>333</x:v>
       </x:c>
       <x:c r="R71"/>
     </x:row>
@@ -6333,7 +6374,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="D72" s="7" t="s">
-        <x:v>321</x:v>
+        <x:v>334</x:v>
       </x:c>
       <x:c r="E72" s="8" t="s">
         <x:v>94</x:v>
@@ -6351,7 +6392,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="J72" s="7" t="s">
-        <x:v>322</x:v>
+        <x:v>335</x:v>
       </x:c>
       <x:c r="K72" s="8" t="s">
         <x:v>140</x:v>
@@ -6370,7 +6411,7 @@
         <x:v>46224</x:v>
       </x:c>
       <x:c r="Q72" s="7" t="s">
-        <x:v>323</x:v>
+        <x:v>336</x:v>
       </x:c>
       <x:c r="R72"/>
     </x:row>
@@ -6382,10 +6423,10 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="C73" s="8" t="s">
-        <x:v>324</x:v>
+        <x:v>337</x:v>
       </x:c>
       <x:c r="D73" s="7" t="s">
-        <x:v>325</x:v>
+        <x:v>338</x:v>
       </x:c>
       <x:c r="E73" s="8" t="s">
         <x:v>95</x:v>
@@ -6397,13 +6438,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H73" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I73" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J73" s="7" t="s">
-        <x:v>326</x:v>
+        <x:v>339</x:v>
       </x:c>
       <x:c r="K73" s="8" t="s">
         <x:v>122</x:v>
@@ -6422,7 +6463,7 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q73" s="7" t="s">
-        <x:v>327</x:v>
+        <x:v>340</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="42" customHeight="1">
@@ -6433,10 +6474,10 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="C74" s="8" t="s">
-        <x:v>328</x:v>
+        <x:v>341</x:v>
       </x:c>
       <x:c r="D74" s="7" t="s">
-        <x:v>329</x:v>
+        <x:v>342</x:v>
       </x:c>
       <x:c r="E74" s="8" t="s">
         <x:v>94</x:v>
@@ -6448,13 +6489,13 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="H74" s="8" t="s">
-        <x:v>152</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="I74" s="8" t="s">
         <x:v>4</x:v>
       </x:c>
       <x:c r="J74" s="7" t="s">
-        <x:v>330</x:v>
+        <x:v>343</x:v>
       </x:c>
       <x:c r="K74" s="8" t="s">
         <x:v>122</x:v>
@@ -6473,105 +6514,105 @@
         <x:v>46225</x:v>
       </x:c>
       <x:c r="Q74" s="7" t="s">
-        <x:v>331</x:v>
+        <x:v>344</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="42" customHeight="1">
-      <x:c r="A75" s="46" t="n">
+      <x:c r="A75" s="8">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="B75" s="46" t="str">
-        <x:v>제작·조립·설치·가공</x:v>
-      </x:c>
-      <x:c r="C75" s="46" t="str">
-        <x:v>템플릿 API</x:v>
-      </x:c>
-      <x:c r="D75" s="45" t="str">
-        <x:v>템플릿 Input 다량 적용 시 보호된 메모리 충돌</x:v>
-      </x:c>
-      <x:c r="E75" s="46" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="F75" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="G75" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H75" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I75" s="46" t="str">
-        <x:v>API 대기</x:v>
-      </x:c>
-      <x:c r="J75" s="45" t="str">
-        <x:v>일부 템플릿에서 Input 항목이 많아지면 적용 중 보호된 메모리 접근 충돌 발생</x:v>
-      </x:c>
-      <x:c r="K75" s="46" t="str">
-        <x:v>API 수정</x:v>
-      </x:c>
-      <x:c r="L75" s="46" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="M75" s="46" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="N75" s="48"/>
-      <x:c r="O75" s="48"/>
-      <x:c r="P75" s="48" t="n">
+      <x:c r="B75" s="8" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C75" s="8" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="D75" s="7" t="s">
+        <x:v>345</x:v>
+      </x:c>
+      <x:c r="E75" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="F75" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="G75" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H75" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I75" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J75" s="7" t="s">
+        <x:v>346</x:v>
+      </x:c>
+      <x:c r="K75" s="8" t="s">
+        <x:v>347</x:v>
+      </x:c>
+      <x:c r="L75" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="M75" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="N75" s="9"/>
+      <x:c r="O75" s="9"/>
+      <x:c r="P75" s="9">
         <x:v>46225</x:v>
       </x:c>
-      <x:c r="Q75" s="45" t="str">
-        <x:v>대량 Input에서도 충돌 없이 템플릿을 적용할 수 있도록 API 안정화 필요</x:v>
+      <x:c r="Q75" s="7" t="s">
+        <x:v>348</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="42" customHeight="1">
-      <x:c r="A76" s="46" t="n">
+      <x:c r="A76" s="8">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B76" s="46" t="str">
-        <x:v>제작·조립·설치·가공</x:v>
-      </x:c>
-      <x:c r="C76" s="46" t="str">
-        <x:v>템플릿 API</x:v>
-      </x:c>
-      <x:c r="D76" s="45" t="str">
-        <x:v>템플릿 텍스트 Bold 적용 API</x:v>
-      </x:c>
-      <x:c r="E76" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="F76" s="46" t="str">
-        <x:v>○</x:v>
-      </x:c>
-      <x:c r="G76" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="H76" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="I76" s="46" t="str">
-        <x:v>API 대기</x:v>
-      </x:c>
-      <x:c r="J76" s="45" t="str">
-        <x:v>템플릿 출력 시 특정 텍스트의 Bold 속성을 코드에서 지정할 수 없음</x:v>
-      </x:c>
-      <x:c r="K76" s="46" t="str">
-        <x:v>API 보강</x:v>
-      </x:c>
-      <x:c r="L76" s="46" t="str">
-        <x:v>X</x:v>
-      </x:c>
-      <x:c r="M76" s="46" t="str">
-        <x:v>O</x:v>
-      </x:c>
-      <x:c r="N76" s="48"/>
-      <x:c r="O76" s="48"/>
-      <x:c r="P76" s="48" t="n">
+      <x:c r="B76" s="8" t="s">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="C76" s="8" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="D76" s="7" t="s">
+        <x:v>349</x:v>
+      </x:c>
+      <x:c r="E76" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="F76" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G76" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="H76" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="I76" s="8" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="J76" s="7" t="s">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="K76" s="8" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="L76" s="8" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="M76" s="8" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="N76" s="9"/>
+      <x:c r="O76" s="9"/>
+      <x:c r="P76" s="9">
         <x:v>46225</x:v>
       </x:c>
-      <x:c r="Q76" s="45" t="str">
-        <x:v>도면 제목·표제부 등 선택 텍스트에 Bold를 적용할 수 있는 API 필요</x:v>
+      <x:c r="Q76" s="7" t="s">
+        <x:v>351</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -6581,28 +6622,51 @@
     <x:mergeCell ref="A3:R3"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="I6:I72">
-    <x:cfRule type="expression" dxfId="10" priority="4">
+    <x:cfRule type="expression" dxfId="17" priority="4">
       <x:formula>$I6="개발 필요"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="9" priority="5">
+    <x:cfRule type="expression" dxfId="16" priority="5">
       <x:formula>$I6="분석 필요"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="8" priority="6">
+    <x:cfRule type="expression" dxfId="15" priority="6">
       <x:formula>$I6="출력 불가"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="7" priority="7">
+    <x:cfRule type="expression" dxfId="14" priority="7">
       <x:formula>$I6="벤더/API 대기"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="I6:I74">
-    <x:cfRule type="expression" dxfId="6" priority="1">
+    <x:cfRule type="expression" dxfId="13" priority="1">
       <x:formula>$I6="완료"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="5" priority="2">
+    <x:cfRule type="expression" dxfId="12" priority="2">
       <x:formula>$I6="실기 검증 대기"</x:formula>
     </x:cfRule>
-    <x:cfRule type="expression" dxfId="4" priority="3">
+    <x:cfRule type="expression" dxfId="11" priority="3">
       <x:formula>$I6="부분 구현"</x:formula>
+    </x:cfRule>
+  </x:conditionalFormatting>
+  <x:conditionalFormatting sqref="I6:I76">
+    <x:cfRule type="expression" dxfId="10" priority="15">
+      <x:formula>$I6="완료"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="9" priority="16">
+      <x:formula>$I6="실기 검증 대기"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="8" priority="17">
+      <x:formula>$I6="부분 구현"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="7" priority="18">
+      <x:formula>$I6="개발 필요"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="6" priority="19">
+      <x:formula>$I6="분석 필요"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="5" priority="20">
+      <x:formula>$I6="출력 불가"</x:formula>
+    </x:cfRule>
+    <x:cfRule type="expression" dxfId="4" priority="21">
+      <x:formula>$I6="API 대기"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:conditionalFormatting sqref="I73:I74">
@@ -6617,29 +6681,6 @@
     </x:cfRule>
     <x:cfRule type="expression" dxfId="0" priority="14">
       <x:formula>$I73="벤더/API 대기"</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="I6:I76">
-    <x:cfRule type="expression" dxfId="11" priority="15">
-      <x:formula>$I6="완료"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="12" priority="16">
-      <x:formula>$I6="실기 검증 대기"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="13" priority="17">
-      <x:formula>$I6="부분 구현"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="14" priority="18">
-      <x:formula>$I6="개발 필요"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="15" priority="19">
-      <x:formula>$I6="분석 필요"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="16" priority="20">
-      <x:formula>$I6="출력 불가"</x:formula>
-    </x:cfRule>
-    <x:cfRule type="expression" dxfId="17" priority="21">
-      <x:formula>$I6="API 대기"</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
   <x:dataValidations count="5">
@@ -6661,7 +6702,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4cba7d535f79497f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e32b0de72de449a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6680,70 +6721,70 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="11" t="s">
-        <x:v>332</x:v>
-      </x:c>
-      <x:c r="B1" s="11"/>
-      <x:c r="C1" s="11"/>
-      <x:c r="D1" s="11"/>
-      <x:c r="E1" s="11"/>
-      <x:c r="F1" s="11"/>
-      <x:c r="G1" s="11"/>
+      <x:c r="A1" s="10" t="s">
+        <x:v>352</x:v>
+      </x:c>
+      <x:c r="B1" s="10"/>
+      <x:c r="C1" s="10"/>
+      <x:c r="D1" s="10"/>
+      <x:c r="E1" s="10"/>
+      <x:c r="F1" s="10"/>
+      <x:c r="G1" s="10"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="28" t="s">
-        <x:v>333</x:v>
-      </x:c>
-      <x:c r="B2" s="28"/>
-      <x:c r="C2" s="28"/>
-      <x:c r="D2" s="28"/>
-      <x:c r="E2" s="28"/>
-      <x:c r="F2" s="28"/>
-      <x:c r="G2" s="28"/>
+      <x:c r="A2" s="41" t="s">
+        <x:v>353</x:v>
+      </x:c>
+      <x:c r="B2" s="41"/>
+      <x:c r="C2" s="41"/>
+      <x:c r="D2" s="41"/>
+      <x:c r="E2" s="41"/>
+      <x:c r="F2" s="41"/>
+      <x:c r="G2" s="41"/>
     </x:row>
     <x:row r="4" ht="15" customHeight="1">
-      <x:c r="A4" s="10" t="s">
-        <x:v>334</x:v>
-      </x:c>
-      <x:c r="B4" s="10"/>
-      <x:c r="C4" s="10"/>
-      <x:c r="D4" s="10"/>
-      <x:c r="E4" s="10"/>
-      <x:c r="F4" s="10"/>
-      <x:c r="G4" s="10"/>
+      <x:c r="A4" s="42" t="s">
+        <x:v>354</x:v>
+      </x:c>
+      <x:c r="B4" s="42"/>
+      <x:c r="C4" s="42"/>
+      <x:c r="D4" s="42"/>
+      <x:c r="E4" s="42"/>
+      <x:c r="F4" s="42"/>
+      <x:c r="G4" s="42"/>
     </x:row>
     <x:row r="5" ht="37.95000076293945" customHeight="1">
       <x:c r="A5" s="2" t="s">
-        <x:v>335</x:v>
+        <x:v>355</x:v>
       </x:c>
       <x:c r="B5" s="2" t="s">
-        <x:v>336</x:v>
+        <x:v>356</x:v>
       </x:c>
       <x:c r="C5" s="2" t="s">
-        <x:v>337</x:v>
+        <x:v>357</x:v>
       </x:c>
       <x:c r="D5" s="2" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="E5" s="2" t="s">
-        <x:v>338</x:v>
+        <x:v>358</x:v>
       </x:c>
       <x:c r="F5" s="2" t="s">
         <x:v>86</x:v>
       </x:c>
       <x:c r="G5" s="2" t="s">
-        <x:v>339</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>340</x:v>
+        <x:v>360</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
-        <x:v>341</x:v>
+        <x:v>361</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>342</x:v>
+        <x:v>362</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
         <x:v>3</x:v>
@@ -6755,18 +6796,18 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>343</x:v>
+        <x:v>363</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
       <x:c r="A7" s="3" t="s">
-        <x:v>344</x:v>
+        <x:v>364</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
-        <x:v>345</x:v>
+        <x:v>365</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>346</x:v>
+        <x:v>366</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
         <x:v>3</x:v>
@@ -6778,18 +6819,18 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>347</x:v>
+        <x:v>367</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
       <x:c r="A8" s="3" t="s">
-        <x:v>348</x:v>
+        <x:v>368</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
-        <x:v>349</x:v>
+        <x:v>369</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>350</x:v>
+        <x:v>370</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
         <x:v>3</x:v>
@@ -6801,18 +6842,18 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>351</x:v>
+        <x:v>371</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
       <x:c r="A9" s="3" t="s">
-        <x:v>352</x:v>
+        <x:v>372</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
-        <x:v>353</x:v>
+        <x:v>373</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>354</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
         <x:v>3</x:v>
@@ -6824,23 +6865,23 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>355</x:v>
+        <x:v>375</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" customHeight="1">
-      <x:c r="A11" s="10" t="s">
-        <x:v>356</x:v>
-      </x:c>
-      <x:c r="B11" s="10"/>
-      <x:c r="C11" s="10"/>
-      <x:c r="D11" s="10"/>
-      <x:c r="E11" s="10"/>
-      <x:c r="F11" s="10"/>
-      <x:c r="G11" s="10"/>
+      <x:c r="A11" s="42" t="s">
+        <x:v>376</x:v>
+      </x:c>
+      <x:c r="B11" s="42"/>
+      <x:c r="C11" s="42"/>
+      <x:c r="D11" s="42"/>
+      <x:c r="E11" s="42"/>
+      <x:c r="F11" s="42"/>
+      <x:c r="G11" s="42"/>
     </x:row>
     <x:row r="12" ht="37.95000076293945" customHeight="1">
       <x:c r="A12" s="2" t="s">
-        <x:v>357</x:v>
+        <x:v>377</x:v>
       </x:c>
       <x:c r="B12" s="2" t="s">
         <x:v>79</x:v>
@@ -6849,21 +6890,21 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="D12" s="2" t="s">
-        <x:v>358</x:v>
+        <x:v>378</x:v>
       </x:c>
       <x:c r="E12" s="2" t="s">
-        <x:v>359</x:v>
+        <x:v>379</x:v>
       </x:c>
       <x:c r="F12" s="2" t="s">
-        <x:v>360</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="G12" s="2" t="s">
-        <x:v>361</x:v>
+        <x:v>381</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
       <x:c r="A13" s="3" t="s">
-        <x:v>286</x:v>
+        <x:v>299</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>94</x:v>
@@ -6872,21 +6913,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>362</x:v>
+        <x:v>382</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>363</x:v>
+        <x:v>383</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>364</x:v>
+        <x:v>384</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
       <x:c r="A14" s="3" t="s">
-        <x:v>289</x:v>
+        <x:v>302</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>94</x:v>
@@ -6895,21 +6936,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>365</x:v>
+        <x:v>385</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>366</x:v>
+        <x:v>386</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>367</x:v>
+        <x:v>387</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
       <x:c r="A15" s="3" t="s">
-        <x:v>292</x:v>
+        <x:v>305</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>94</x:v>
@@ -6918,21 +6959,21 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>368</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>368</x:v>
+        <x:v>388</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>294</x:v>
+        <x:v>307</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
       <x:c r="A16" s="3" t="s">
-        <x:v>151</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>94</x:v>
@@ -6941,16 +6982,16 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>369</x:v>
+        <x:v>389</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>370</x:v>
+        <x:v>390</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
-        <x:v>371</x:v>
+        <x:v>391</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>372</x:v>
+        <x:v>392</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36" customHeight="1">
@@ -6961,24 +7002,24 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>374</x:v>
+        <x:v>394</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>375</x:v>
+        <x:v>395</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>377</x:v>
+        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
       <x:c r="A18" s="3" t="s">
-        <x:v>295</x:v>
+        <x:v>308</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>94</x:v>
@@ -6987,16 +7028,16 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>378</x:v>
+        <x:v>398</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>379</x:v>
+        <x:v>399</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>380</x:v>
+        <x:v>400</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
@@ -7007,19 +7048,19 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>381</x:v>
+        <x:v>401</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>382</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>377</x:v>
+        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
@@ -7030,31 +7071,31 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>383</x:v>
+        <x:v>403</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>382</x:v>
+        <x:v>402</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>377</x:v>
+        <x:v>397</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15" customHeight="1">
-      <x:c r="A22" s="10" t="s">
-        <x:v>384</x:v>
-      </x:c>
-      <x:c r="B22" s="10"/>
-      <x:c r="C22" s="10"/>
-      <x:c r="D22" s="10"/>
-      <x:c r="E22" s="10"/>
-      <x:c r="F22" s="10"/>
-      <x:c r="G22" s="10"/>
+      <x:c r="A22" s="42" t="s">
+        <x:v>404</x:v>
+      </x:c>
+      <x:c r="B22" s="42"/>
+      <x:c r="C22" s="42"/>
+      <x:c r="D22" s="42"/>
+      <x:c r="E22" s="42"/>
+      <x:c r="F22" s="42"/>
+      <x:c r="G22" s="42"/>
     </x:row>
     <x:row r="23" ht="37.95000076293945" customHeight="1">
       <x:c r="A23" s="2" t="s">
@@ -7067,67 +7108,67 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="D23" s="2" t="s">
-        <x:v>385</x:v>
+        <x:v>405</x:v>
       </x:c>
       <x:c r="E23" s="2" t="s">
-        <x:v>386</x:v>
+        <x:v>406</x:v>
       </x:c>
       <x:c r="F23" s="2" t="s">
-        <x:v>360</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="G23" s="2" t="s">
-        <x:v>339</x:v>
+        <x:v>359</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="3" t="s">
-        <x:v>387</x:v>
+        <x:v>407</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>94</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>388</x:v>
+        <x:v>408</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>389</x:v>
+        <x:v>409</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>390</x:v>
+        <x:v>410</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
       <x:c r="A25" s="3" t="s">
-        <x:v>391</x:v>
+        <x:v>411</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>94</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>392</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>393</x:v>
+        <x:v>413</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>394</x:v>
+        <x:v>414</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
       <x:c r="A26" s="3" t="s">
-        <x:v>395</x:v>
+        <x:v>415</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>120</x:v>
@@ -7136,67 +7177,67 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>392</x:v>
+        <x:v>412</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
+        <x:v>416</x:v>
+      </x:c>
+      <x:c r="F26" s="3" t="s">
         <x:v>396</x:v>
       </x:c>
-      <x:c r="F26" s="3" t="s">
-        <x:v>376</x:v>
-      </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>397</x:v>
+        <x:v>417</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="36" customHeight="1">
       <x:c r="A27" s="3" t="s">
-        <x:v>398</x:v>
+        <x:v>418</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>94</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>399</x:v>
+        <x:v>419</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>400</x:v>
+        <x:v>420</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>401</x:v>
+        <x:v>421</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
       <x:c r="A28" s="3" t="s">
-        <x:v>402</x:v>
+        <x:v>422</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>94</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>403</x:v>
+        <x:v>423</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>404</x:v>
+        <x:v>424</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>405</x:v>
+        <x:v>425</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="36" customHeight="1">
       <x:c r="A29" s="3" t="s">
-        <x:v>406</x:v>
+        <x:v>426</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>94</x:v>
@@ -7205,21 +7246,21 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>407</x:v>
+        <x:v>427</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>408</x:v>
+        <x:v>428</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>409</x:v>
+        <x:v>429</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="36" customHeight="1">
       <x:c r="A30" s="3" t="s">
-        <x:v>410</x:v>
+        <x:v>430</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>94</x:v>
@@ -7228,21 +7269,21 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>411</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>412</x:v>
+        <x:v>432</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>409</x:v>
+        <x:v>429</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="36" customHeight="1">
       <x:c r="A31" s="3" t="s">
-        <x:v>413</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>94</x:v>
@@ -7251,16 +7292,16 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>414</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>415</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
-        <x:v>416</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>417</x:v>
+        <x:v>437</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="36" customHeight="1">
@@ -7271,24 +7312,24 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>373</x:v>
+        <x:v>393</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>418</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>419</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>420</x:v>
+        <x:v>440</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
       <x:c r="A33" s="3" t="s">
-        <x:v>248</x:v>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>95</x:v>
@@ -7297,13 +7338,13 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>421</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>422</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
-        <x:v>423</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
         <x:v>80</x:v>
@@ -7311,7 +7352,7 @@
     </x:row>
     <x:row r="34" ht="36" customHeight="1">
       <x:c r="A34" s="3" t="s">
-        <x:v>424</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>95</x:v>
@@ -7320,28 +7361,28 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>425</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>426</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
         <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
-      <x:c r="A36" s="29" t="s">
-        <x:v>427</x:v>
-      </x:c>
-      <x:c r="B36" s="29"/>
-      <x:c r="C36" s="29"/>
-      <x:c r="D36" s="29"/>
-      <x:c r="E36" s="29"/>
-      <x:c r="F36" s="29"/>
-      <x:c r="G36" s="29"/>
+      <x:c r="A36" s="31" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="B36" s="31"/>
+      <x:c r="C36" s="31"/>
+      <x:c r="D36" s="31"/>
+      <x:c r="E36" s="31"/>
+      <x:c r="F36" s="31"/>
+      <x:c r="G36" s="31"/>
     </x:row>
     <x:row r="37" ht="37.95000076293945" customHeight="1">
       <x:c r="A37" s="6" t="s">
@@ -7354,21 +7395,21 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="D37" s="6" t="s">
-        <x:v>428</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="E37" s="6" t="s">
-        <x:v>429</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="F37" s="6" t="s">
-        <x:v>360</x:v>
+        <x:v>380</x:v>
       </x:c>
       <x:c r="G37" s="6" t="s">
-        <x:v>361</x:v>
+        <x:v>381</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="36" customHeight="1">
       <x:c r="A38" s="7" t="s">
-        <x:v>430</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="B38" s="7" t="s">
         <x:v>94</x:v>
@@ -7377,21 +7418,21 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="D38" s="7" t="s">
-        <x:v>431</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="E38" s="7" t="s">
-        <x:v>432</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F38" s="7" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G38" s="7" t="s">
-        <x:v>433</x:v>
+        <x:v>453</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="36" customHeight="1">
       <x:c r="A39" s="7" t="s">
-        <x:v>434</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B39" s="7" t="s">
         <x:v>120</x:v>
@@ -7400,21 +7441,21 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="D39" s="7" t="s">
-        <x:v>435</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="E39" s="7" t="s">
-        <x:v>436</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="F39" s="7" t="s">
-        <x:v>376</x:v>
+        <x:v>396</x:v>
       </x:c>
       <x:c r="G39" s="7" t="s">
-        <x:v>437</x:v>
+        <x:v>457</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="36" customHeight="1">
       <x:c r="A40" s="7" t="s">
-        <x:v>438</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="B40" s="7" t="s">
         <x:v>95</x:v>
@@ -7423,21 +7464,21 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D40" s="7" t="s">
-        <x:v>439</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="E40" s="7" t="s">
-        <x:v>440</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="F40" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G40" s="7" t="s">
-        <x:v>441</x:v>
+        <x:v>461</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="36" customHeight="1">
       <x:c r="A41" s="7" t="s">
-        <x:v>442</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="B41" s="7" t="s">
         <x:v>94</x:v>
@@ -7446,50 +7487,50 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="D41" s="7" t="s">
-        <x:v>443</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="E41" s="7" t="s">
-        <x:v>444</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="F41" s="7" t="s">
         <x:v>122</x:v>
       </x:c>
       <x:c r="G41" s="7" t="s">
-        <x:v>445</x:v>
+        <x:v>465</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="25.950000762939453" customHeight="1">
-      <x:c r="A43" s="30" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="B43" s="31"/>
-      <x:c r="C43" s="31"/>
-      <x:c r="D43" s="31"/>
-      <x:c r="E43" s="31"/>
-      <x:c r="F43" s="31"/>
-      <x:c r="G43" s="32"/>
+      <x:c r="A43" s="32" t="s">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="B43" s="33"/>
+      <x:c r="C43" s="33"/>
+      <x:c r="D43" s="33"/>
+      <x:c r="E43" s="33"/>
+      <x:c r="F43" s="33"/>
+      <x:c r="G43" s="34"/>
     </x:row>
     <x:row r="44" ht="25.950000762939453" customHeight="1">
-      <x:c r="A44" s="33" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="B44" s="34"/>
-      <x:c r="C44" s="34"/>
-      <x:c r="D44" s="34"/>
-      <x:c r="E44" s="34"/>
-      <x:c r="F44" s="34"/>
-      <x:c r="G44" s="35"/>
+      <x:c r="A44" s="35" t="s">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="B44" s="36"/>
+      <x:c r="C44" s="36"/>
+      <x:c r="D44" s="36"/>
+      <x:c r="E44" s="36"/>
+      <x:c r="F44" s="36"/>
+      <x:c r="G44" s="37"/>
     </x:row>
     <x:row r="45" ht="25.950000762939453" customHeight="1">
-      <x:c r="A45" s="36" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="B45" s="37"/>
-      <x:c r="C45" s="37"/>
-      <x:c r="D45" s="37"/>
-      <x:c r="E45" s="37"/>
-      <x:c r="F45" s="37"/>
-      <x:c r="G45" s="38"/>
+      <x:c r="A45" s="38" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="B45" s="39"/>
+      <x:c r="C45" s="39"/>
+      <x:c r="D45" s="39"/>
+      <x:c r="E45" s="39"/>
+      <x:c r="F45" s="39"/>
+      <x:c r="G45" s="40"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>